<commit_message>
Gráfico interactivo de consenso: seguimiento + pronóstico + votación, registro en Consenso.xlsx y consolidación por rondas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FeXNtAXpW6U6SWYhWp9Fpb
</commit_message>
<xml_diff>
--- a/Seguimiento/Seguimiento_Aportes.xlsx
+++ b/Seguimiento/Seguimiento_Aportes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\co33377228\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\co33377228\Documents\2026\Objetivos\Consenso\Consenso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7C4FC9-46C9-44D6-BD56-68C80BDFF911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{257A6F82-BEE8-46AC-AC34-3AF4F90911B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{08D9150E-D939-445D-91CB-DD8FC739B0D9}"/>
   </bookViews>
@@ -48,10 +48,25 @@
     <t>SIN</t>
   </si>
   <si>
+    <t>Fecha de inicio graficos</t>
+  </si>
+  <si>
+    <t>Fecha de fin Graficos</t>
+  </si>
+  <si>
+    <t>fecha</t>
+  </si>
+  <si>
+    <t>activa</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
     <t>Cuenca 1</t>
   </si>
   <si>
-    <t>Ceunca 2</t>
+    <t>Cuenca 2</t>
   </si>
   <si>
     <t>Cuenca 3</t>
@@ -67,21 +82,6 @@
   </si>
   <si>
     <t>Cuenca 7</t>
-  </si>
-  <si>
-    <t>Fecha de inicio graficos</t>
-  </si>
-  <si>
-    <t>Fecha de fin Graficos</t>
-  </si>
-  <si>
-    <t>fecha</t>
-  </si>
-  <si>
-    <t>activa</t>
-  </si>
-  <si>
-    <t>no</t>
   </si>
 </sst>
 </file>
@@ -458,9 +458,31 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="7">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{A5D53130-2C34-4F83-99E3-10E8342DE54C}">
+  <we:reference id="wa200007447" version="1.1.6.7" store="es-ES" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200007447" version="1.1.6.7" store="WA200007447" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="hello" value="{&quot;name&quot;:&quot;hello&quot;,&quot;code&quot;:&quot;def hello(name):\n    \&quot;\&quot;\&quot; Returns a greeting. \&quot;\&quot;\&quot;\n    return f\&quot;Hello {name}!\&quot;\n\n\n\n\n    \n# Code MUST be a function!\n# Save creates an Excel function\n# e.g. =HELLO(\&quot;World\&quot;)\n# Click 📖 to see full docs\n# Try examples in Functions tab&quot;,&quot;options&quot;:{},&quot;signature&quot;:&quot;HELLO(name)&quot;,&quot;description&quot;:&quot;Returns a greeting.&quot;,&quot;resultLine&quot;:&quot;\n\nresult = hello(**{k: v for k, v in [(\&quot;name\&quot;, arg1 if arg1 != \&quot;__OMITTED__\&quot; else None)] if v is not None})&quot;,&quot;timestamp&quot;:&quot;2026-07-01T13:58:02.685Z&quot;,&quot;parameters&quot;:[{&quot;name&quot;:&quot;name&quot;,&quot;optional&quot;:false}],&quot;imports&quot;:[],&quot;external_packages&quot;:[],&quot;isUserDefined&quot;:true}"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEEDB5BB-C780-4A2C-BE1D-ED8FE9585C5C}">
-  <dimension ref="A1:I298"/>
+  <dimension ref="A1:I302"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -471,25 +493,25 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -6357,7 +6379,7 @@
         <v>46.952181896944829</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A257" s="1">
         <v>46278</v>
       </c>
@@ -6380,7 +6402,7 @@
         <v>41.373773461012306</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A258" s="1">
         <v>46279</v>
       </c>
@@ -6403,7 +6425,7 @@
         <v>39.116762881896946</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A259" s="1">
         <v>46280</v>
       </c>
@@ -6426,7 +6448,7 @@
         <v>37.916225034199726</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A260" s="1">
         <v>46281</v>
       </c>
@@ -6449,7 +6471,7 @@
         <v>37.245655175558596</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A261" s="1">
         <v>46282</v>
       </c>
@@ -6472,7 +6494,7 @@
         <v>36.03266570907433</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A262" s="1">
         <v>46283</v>
       </c>
@@ -6495,7 +6517,7 @@
         <v>34.866785544915643</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A263" s="1">
         <v>46284</v>
       </c>
@@ -6518,7 +6540,7 @@
         <v>34.521146192430464</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A264" s="1">
         <v>46285</v>
       </c>
@@ -6541,7 +6563,7 @@
         <v>34.838802279981763</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A265" s="1">
         <v>46286</v>
       </c>
@@ -6564,7 +6586,7 @@
         <v>35.458411491108073</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A266" s="1">
         <v>46287</v>
       </c>
@@ -6587,7 +6609,7 @@
         <v>34.324023210214314</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A267" s="1">
         <v>46288</v>
       </c>
@@ -6609,8 +6631,14 @@
       <c r="G267">
         <v>34.660634017327865</v>
       </c>
-    </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H267">
+        <v>40.657605407240148</v>
+      </c>
+      <c r="I267">
+        <v>58.301082445356954</v>
+      </c>
+    </row>
+    <row r="268" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A268" s="1">
         <v>46289</v>
       </c>
@@ -6632,8 +6660,14 @@
       <c r="G268">
         <v>33.826530141358866</v>
       </c>
-    </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H268">
+        <v>49.55948111745694</v>
+      </c>
+      <c r="I268">
+        <v>95.230514612694478</v>
+      </c>
+    </row>
+    <row r="269" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A269" s="1">
         <v>46290</v>
       </c>
@@ -6655,8 +6689,14 @@
       <c r="G269">
         <v>38.347140036479708</v>
       </c>
-    </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H269">
+        <v>46.563657561133986</v>
+      </c>
+      <c r="I269">
+        <v>73.631506352993995</v>
+      </c>
+    </row>
+    <row r="270" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A270" s="1">
         <v>46291</v>
       </c>
@@ -6678,8 +6718,14 @@
       <c r="G270">
         <v>37.313816142270859</v>
       </c>
-    </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H270">
+        <v>35.265123005858825</v>
+      </c>
+      <c r="I270">
+        <v>67.1680437309182</v>
+      </c>
+    </row>
+    <row r="271" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A271" s="1">
         <v>46292</v>
       </c>
@@ -6701,8 +6747,14 @@
       <c r="G271">
         <v>45.346786548107623</v>
       </c>
-    </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H271">
+        <v>35.436312923362991</v>
+      </c>
+      <c r="I271">
+        <v>96.107466827749988</v>
+      </c>
+    </row>
+    <row r="272" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A272" s="1">
         <v>46293</v>
       </c>
@@ -6724,8 +6776,14 @@
       <c r="G272">
         <v>81.715805927952573</v>
       </c>
-    </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H272">
+        <v>349.5698115435132</v>
+      </c>
+      <c r="I272">
+        <v>106.6308934084161</v>
+      </c>
+    </row>
+    <row r="273" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A273" s="1">
         <v>46294</v>
       </c>
@@ -6747,8 +6805,14 @@
       <c r="G273">
         <v>53.088072685818524</v>
       </c>
-    </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H273">
+        <v>75.494753619338553</v>
+      </c>
+      <c r="I273">
+        <v>100.55718732636498</v>
+      </c>
+    </row>
+    <row r="274" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A274" s="1">
         <v>46295</v>
       </c>
@@ -6770,8 +6834,14 @@
       <c r="G274">
         <v>44.275296306429553</v>
       </c>
-    </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H274">
+        <v>41.25677011850474</v>
+      </c>
+      <c r="I274">
+        <v>76.749558673191359</v>
+      </c>
+    </row>
+    <row r="275" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A275" s="1">
         <v>46296</v>
       </c>
@@ -6793,8 +6863,14 @@
       <c r="G275">
         <v>71.953264166001603</v>
       </c>
-    </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H275">
+        <v>43.707611152976646</v>
+      </c>
+      <c r="I275">
+        <v>98.175507727219511</v>
+      </c>
+    </row>
+    <row r="276" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A276" s="1">
         <v>46297</v>
       </c>
@@ -6816,8 +6892,14 @@
       <c r="G276">
         <v>46.344505067837197</v>
       </c>
-    </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H276">
+        <v>165.23377346744869</v>
+      </c>
+      <c r="I276">
+        <v>83.106243155116985</v>
+      </c>
+    </row>
+    <row r="277" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A277" s="1">
         <v>46298</v>
       </c>
@@ -6839,8 +6921,14 @@
       <c r="G277">
         <v>38.187954349561053</v>
       </c>
-    </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H277">
+        <v>108.22384587660959</v>
+      </c>
+      <c r="I277">
+        <v>61.503626334976637</v>
+      </c>
+    </row>
+    <row r="278" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A278" s="1">
         <v>46299</v>
       </c>
@@ -6862,8 +6950,14 @@
       <c r="G278">
         <v>36.153272266560258</v>
       </c>
-    </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H278">
+        <v>31.830542904885167</v>
+      </c>
+      <c r="I278">
+        <v>61.028018316920239</v>
+      </c>
+    </row>
+    <row r="279" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A279" s="1">
         <v>46300</v>
       </c>
@@ -6885,8 +6979,14 @@
       <c r="G279">
         <v>34.595246568236234</v>
       </c>
-    </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H279">
+        <v>38.101634939877471</v>
+      </c>
+      <c r="I279">
+        <v>77.173658929887239</v>
+      </c>
+    </row>
+    <row r="280" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A280" s="1">
         <v>46301</v>
       </c>
@@ -6908,8 +7008,14 @@
       <c r="G280">
         <v>37.096249002394252</v>
       </c>
-    </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H280">
+        <v>31.450476720946241</v>
+      </c>
+      <c r="I280">
+        <v>108.66391612541048</v>
+      </c>
+    </row>
+    <row r="281" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A281" s="1">
         <v>46302</v>
       </c>
@@ -6931,8 +7037,14 @@
       <c r="G281">
         <v>39.820304788507585</v>
       </c>
-    </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H281">
+        <v>18.813276104976907</v>
+      </c>
+      <c r="I281">
+        <v>112.91935628696767</v>
+      </c>
+    </row>
+    <row r="282" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A282" s="1">
         <v>46303</v>
       </c>
@@ -6954,8 +7066,14 @@
       <c r="G282">
         <v>45.090108619313654</v>
       </c>
-    </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H282">
+        <v>37.626552209953815</v>
+      </c>
+      <c r="I282">
+        <v>101.20437984221023</v>
+      </c>
+    </row>
+    <row r="283" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A283" s="1">
         <v>46304</v>
       </c>
@@ -6977,8 +7095,14 @@
       <c r="G283">
         <v>52.40504094173982</v>
       </c>
-    </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H283">
+        <v>62.710920349923015</v>
+      </c>
+      <c r="I283">
+        <v>124.90968474217883</v>
+      </c>
+    </row>
+    <row r="284" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A284" s="1">
         <v>46305</v>
       </c>
@@ -7000,8 +7124,14 @@
       <c r="G284">
         <v>42.897040981644054</v>
       </c>
-    </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H284">
+        <v>87.700271943907509</v>
+      </c>
+      <c r="I284">
+        <v>184.43578300207889</v>
+      </c>
+    </row>
+    <row r="285" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A285" s="1">
         <v>46306</v>
       </c>
@@ -7023,8 +7153,14 @@
       <c r="G285">
         <v>40.023810893854751</v>
       </c>
-    </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H285">
+        <v>43.897644244946115</v>
+      </c>
+      <c r="I285">
+        <v>132.39425302632944</v>
+      </c>
+    </row>
+    <row r="286" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A286" s="1">
         <v>46307</v>
       </c>
@@ -7046,8 +7182,14 @@
       <c r="G286">
         <v>65.871010614525133</v>
       </c>
-    </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H286">
+        <v>87.605255397922761</v>
+      </c>
+      <c r="I286">
+        <v>107.3121880740923</v>
+      </c>
+    </row>
+    <row r="287" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A287" s="1">
         <v>46308</v>
       </c>
@@ -7069,8 +7211,14 @@
       <c r="G287">
         <v>66.590413288108536</v>
       </c>
-    </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H287">
+        <v>81.144130270960986</v>
+      </c>
+      <c r="I287">
+        <v>134.22158909570399</v>
+      </c>
+    </row>
+    <row r="288" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A288" s="1">
         <v>46309</v>
       </c>
@@ -7092,8 +7240,14 @@
       <c r="G288">
         <v>48.310028411811651</v>
       </c>
-    </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H288">
+        <v>68.791979292945854</v>
+      </c>
+      <c r="I288">
+        <v>156.37490993675175</v>
+      </c>
+    </row>
+    <row r="289" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A289" s="1">
         <v>46310</v>
       </c>
@@ -7115,8 +7269,14 @@
       <c r="G289">
         <v>43.319815522745415</v>
       </c>
-    </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H289">
+        <v>74.873038235968693</v>
+      </c>
+      <c r="I289">
+        <v>155.82420591584435</v>
+      </c>
+    </row>
+    <row r="290" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A290" s="1">
         <v>46311</v>
       </c>
@@ -7132,14 +7292,17 @@
       <c r="E290">
         <v>64.632675816539262</v>
       </c>
-      <c r="F290">
-        <v>0</v>
-      </c>
       <c r="G290">
         <v>46.872833200319242</v>
       </c>
-    </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H290">
+        <v>43.707611152976646</v>
+      </c>
+      <c r="I290">
+        <v>115.04707636774627</v>
+      </c>
+    </row>
+    <row r="291" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A291" s="1">
         <v>46312</v>
       </c>
@@ -7161,8 +7324,14 @@
       <c r="G291">
         <v>42.68155327214685</v>
       </c>
-    </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H291">
+        <v>49.978703187968947</v>
+      </c>
+      <c r="I291">
+        <v>90.490683435466224</v>
+      </c>
+    </row>
+    <row r="292" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A292" s="1">
         <v>46313</v>
       </c>
@@ -7184,8 +7353,14 @@
       <c r="G292">
         <v>39.836181644054278</v>
       </c>
-    </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H292">
+        <v>49.88368664198422</v>
+      </c>
+      <c r="I292">
+        <v>78.850802993559782</v>
+      </c>
+    </row>
+    <row r="293" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A293" s="1">
         <v>46314</v>
       </c>
@@ -7207,8 +7382,14 @@
       <c r="G293">
         <v>39.64196169193935</v>
       </c>
-    </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H293">
+        <v>31.165427082992043</v>
+      </c>
+      <c r="I293">
+        <v>77.574170945092618</v>
+      </c>
+    </row>
+    <row r="294" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A294" s="1">
         <v>46315</v>
       </c>
@@ -7230,8 +7411,14 @@
       <c r="G294">
         <v>38.537414445331208</v>
       </c>
-    </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H294">
+        <v>37.246486026014885</v>
+      </c>
+      <c r="I294">
+        <v>75.771866876668398</v>
+      </c>
+    </row>
+    <row r="295" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A295" s="1">
         <v>46316</v>
       </c>
@@ -7253,8 +7440,14 @@
       <c r="G295">
         <v>60.074488866719875</v>
       </c>
-    </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H295">
+        <v>30.975393991022582</v>
+      </c>
+      <c r="I295">
+        <v>90.665907442118581</v>
+      </c>
+    </row>
+    <row r="296" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A296" s="1">
         <v>46317</v>
       </c>
@@ -7276,8 +7469,14 @@
       <c r="G296">
         <v>54.253403990422989</v>
       </c>
-    </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H296">
+        <v>31.070410537007316</v>
+      </c>
+      <c r="I296">
+        <v>77.799458953645654</v>
+      </c>
+    </row>
+    <row r="297" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A297" s="1">
         <v>46318</v>
       </c>
@@ -7299,8 +7498,14 @@
       <c r="G297">
         <v>43.574318515562652</v>
       </c>
-    </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H297">
+        <v>31.070410537007316</v>
+      </c>
+      <c r="I297">
+        <v>84.783387218789514</v>
+      </c>
+    </row>
+    <row r="298" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A298" s="1">
         <v>46319</v>
       </c>
@@ -7321,6 +7526,128 @@
       </c>
       <c r="G298">
         <v>47.863775937749402</v>
+      </c>
+      <c r="H298">
+        <v>18.718259558992173</v>
+      </c>
+      <c r="I298">
+        <v>85.309059238746585</v>
+      </c>
+    </row>
+    <row r="299" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A299" s="1">
+        <v>46320</v>
+      </c>
+      <c r="B299">
+        <v>52.761801762684456</v>
+      </c>
+      <c r="C299">
+        <v>95.347634934497819</v>
+      </c>
+      <c r="D299">
+        <v>72.922874074074073</v>
+      </c>
+      <c r="E299">
+        <v>49.90312543432939</v>
+      </c>
+      <c r="F299">
+        <v>18.525535332785541</v>
+      </c>
+      <c r="G299">
+        <v>50.247543176376695</v>
+      </c>
+      <c r="H299">
+        <v>18.908292650961638</v>
+      </c>
+      <c r="I299">
+        <v>52.492105992855507</v>
+      </c>
+    </row>
+    <row r="300" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A300" s="1">
+        <v>46321</v>
+      </c>
+      <c r="B300">
+        <v>62.75562580149586</v>
+      </c>
+      <c r="C300">
+        <v>81.360267248908286</v>
+      </c>
+      <c r="D300">
+        <v>75.982399999999998</v>
+      </c>
+      <c r="E300">
+        <v>48.999975816539262</v>
+      </c>
+      <c r="F300">
+        <v>56.935988249794576</v>
+      </c>
+      <c r="G300">
+        <v>49.577641739824429</v>
+      </c>
+      <c r="H300">
+        <v>25.179384685953938</v>
+      </c>
+      <c r="I300">
+        <v>79.000994999261792</v>
+      </c>
+    </row>
+    <row r="301" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A301" s="1">
+        <v>46322</v>
+      </c>
+      <c r="B301">
+        <v>68.977988465736814</v>
+      </c>
+      <c r="C301">
+        <v>78.864288209606983</v>
+      </c>
+      <c r="D301">
+        <v>80.378903703703713</v>
+      </c>
+      <c r="E301">
+        <v>44.024442043085479</v>
+      </c>
+      <c r="F301">
+        <v>43.784754971240751</v>
+      </c>
+      <c r="G301">
+        <v>53.744433519553084</v>
+      </c>
+      <c r="H301">
+        <v>25.084368139969211</v>
+      </c>
+      <c r="I301">
+        <v>71.741714723664245</v>
+      </c>
+    </row>
+    <row r="302" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A302" s="1">
+        <v>46323</v>
+      </c>
+      <c r="B302">
+        <v>58.991804010511416</v>
+      </c>
+      <c r="C302">
+        <v>78.864288209606983</v>
+      </c>
+      <c r="D302">
+        <v>80.378903703703713</v>
+      </c>
+      <c r="E302">
+        <v>44.024442043085479</v>
+      </c>
+      <c r="F302">
+        <v>43.784754971240751</v>
+      </c>
+      <c r="G302">
+        <v>51.008846089385472</v>
+      </c>
+      <c r="H302">
+        <v>15.39268044952656</v>
+      </c>
+      <c r="I302">
+        <v>95.321859618881149</v>
       </c>
     </row>
   </sheetData>
@@ -7342,32 +7669,32 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1">
-        <v>46318</v>
+        <v>46288</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1">
-        <v>46317</v>
+        <v>46324</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>